<commit_message>
Agregar cedula a administracion de usuarios
</commit_message>
<xml_diff>
--- a/plantillas/plantilla_cuentas_docentes.xlsx
+++ b/plantillas/plantilla_cuentas_docentes.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Docentes" sheetId="1" r:id="Ra415354427c349ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R5f211504e4634b72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Docentes" sheetId="1" r:id="Rd4678a83dd1348db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R8c44556a6b2a4e35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +17,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="@"/>
   </x:numFmts>
-  <x:fonts count="6">
+  <x:fonts count="7">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -51,8 +51,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -99,6 +105,11 @@
         <x:fgColor rgb="FFF2F7FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF087F5B"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="3">
     <x:border/>
@@ -134,7 +145,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="26">
+  <x:cellXfs count="30">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -183,6 +194,12 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -389,6 +406,7 @@
     <x:col min="2" max="2" width="42" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="34" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -404,306 +422,506 @@
       <x:c r="D1" s="24" t="str">
         <x:v>Unidad</x:v>
       </x:c>
+      <x:c r="E1" s="29" t="str">
+        <x:v>Cédula</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="23" customHeight="1">
       <x:c r="A2" s="9" t="str"/>
       <x:c r="B2" s="10" t="str"/>
       <x:c r="C2" s="11" t="str"/>
       <x:c r="D2" s="25"/>
+      <x:c r="E2" s="26"/>
     </x:row>
     <x:row r="3" ht="23" customHeight="1">
       <x:c r="A3" s="9" t="str"/>
       <x:c r="B3" s="10" t="str"/>
       <x:c r="C3" s="11" t="str"/>
       <x:c r="D3" s="25"/>
+      <x:c r="E3" s="26"/>
     </x:row>
     <x:row r="4" ht="23" customHeight="1">
       <x:c r="A4" s="9" t="str"/>
       <x:c r="B4" s="10" t="str"/>
       <x:c r="C4" s="11" t="str"/>
       <x:c r="D4" s="25"/>
+      <x:c r="E4" s="26"/>
     </x:row>
     <x:row r="5" ht="23" customHeight="1">
       <x:c r="A5" s="9" t="str"/>
       <x:c r="B5" s="10" t="str"/>
       <x:c r="C5" s="11" t="str"/>
       <x:c r="D5" s="25"/>
+      <x:c r="E5" s="26"/>
     </x:row>
     <x:row r="6" ht="23" customHeight="1">
       <x:c r="A6" s="9" t="str"/>
       <x:c r="B6" s="10" t="str"/>
       <x:c r="C6" s="11" t="str"/>
       <x:c r="D6" s="25"/>
+      <x:c r="E6" s="26"/>
     </x:row>
     <x:row r="7" ht="23" customHeight="1">
       <x:c r="A7" s="9" t="str"/>
       <x:c r="B7" s="10" t="str"/>
       <x:c r="C7" s="11" t="str"/>
       <x:c r="D7" s="25"/>
+      <x:c r="E7" s="26"/>
     </x:row>
     <x:row r="8" ht="23" customHeight="1">
       <x:c r="A8" s="9" t="str"/>
       <x:c r="B8" s="10" t="str"/>
       <x:c r="C8" s="11" t="str"/>
       <x:c r="D8" s="25"/>
+      <x:c r="E8" s="26"/>
     </x:row>
     <x:row r="9" ht="23" customHeight="1">
       <x:c r="A9" s="9" t="str"/>
       <x:c r="B9" s="10" t="str"/>
       <x:c r="C9" s="11" t="str"/>
       <x:c r="D9" s="25"/>
+      <x:c r="E9" s="26"/>
     </x:row>
     <x:row r="10" ht="23" customHeight="1">
       <x:c r="A10" s="9" t="str"/>
       <x:c r="B10" s="10" t="str"/>
       <x:c r="C10" s="11" t="str"/>
       <x:c r="D10" s="25"/>
+      <x:c r="E10" s="26"/>
     </x:row>
     <x:row r="11" ht="23" customHeight="1">
       <x:c r="A11" s="9" t="str"/>
       <x:c r="B11" s="10" t="str"/>
       <x:c r="C11" s="11" t="str"/>
       <x:c r="D11" s="25"/>
+      <x:c r="E11" s="26"/>
     </x:row>
     <x:row r="12" ht="23" customHeight="1">
       <x:c r="A12" s="9" t="str"/>
       <x:c r="B12" s="10" t="str"/>
       <x:c r="C12" s="11" t="str"/>
       <x:c r="D12" s="25"/>
+      <x:c r="E12" s="26"/>
     </x:row>
     <x:row r="13" ht="23" customHeight="1">
       <x:c r="A13" s="9" t="str"/>
       <x:c r="B13" s="10" t="str"/>
       <x:c r="C13" s="11" t="str"/>
       <x:c r="D13" s="25"/>
+      <x:c r="E13" s="26"/>
     </x:row>
     <x:row r="14" ht="23" customHeight="1">
       <x:c r="A14" s="9" t="str"/>
       <x:c r="B14" s="10" t="str"/>
       <x:c r="C14" s="11" t="str"/>
       <x:c r="D14" s="25"/>
+      <x:c r="E14" s="26"/>
     </x:row>
     <x:row r="15" ht="23" customHeight="1">
       <x:c r="A15" s="9" t="str"/>
       <x:c r="B15" s="10" t="str"/>
       <x:c r="C15" s="11" t="str"/>
       <x:c r="D15" s="25"/>
+      <x:c r="E15" s="26"/>
     </x:row>
     <x:row r="16" ht="23" customHeight="1">
       <x:c r="A16" s="9" t="str"/>
       <x:c r="B16" s="10" t="str"/>
       <x:c r="C16" s="11" t="str"/>
       <x:c r="D16" s="25"/>
+      <x:c r="E16" s="26"/>
     </x:row>
     <x:row r="17" ht="23" customHeight="1">
       <x:c r="A17" s="9" t="str"/>
       <x:c r="B17" s="10" t="str"/>
       <x:c r="C17" s="11" t="str"/>
       <x:c r="D17" s="25"/>
+      <x:c r="E17" s="26"/>
     </x:row>
     <x:row r="18" ht="23" customHeight="1">
       <x:c r="A18" s="9" t="str"/>
       <x:c r="B18" s="10" t="str"/>
       <x:c r="C18" s="11" t="str"/>
       <x:c r="D18" s="25"/>
+      <x:c r="E18" s="26"/>
     </x:row>
     <x:row r="19" ht="23" customHeight="1">
       <x:c r="A19" s="9" t="str"/>
       <x:c r="B19" s="10" t="str"/>
       <x:c r="C19" s="11" t="str"/>
       <x:c r="D19" s="25"/>
+      <x:c r="E19" s="26"/>
     </x:row>
     <x:row r="20" ht="23" customHeight="1">
       <x:c r="A20" s="9" t="str"/>
       <x:c r="B20" s="10" t="str"/>
       <x:c r="C20" s="11" t="str"/>
       <x:c r="D20" s="25"/>
+      <x:c r="E20" s="26"/>
     </x:row>
     <x:row r="21" ht="23" customHeight="1">
       <x:c r="A21" s="9" t="str"/>
       <x:c r="B21" s="10" t="str"/>
       <x:c r="C21" s="11" t="str"/>
       <x:c r="D21" s="25"/>
+      <x:c r="E21" s="26"/>
     </x:row>
     <x:row r="22" ht="23" customHeight="1">
       <x:c r="A22" s="9" t="str"/>
       <x:c r="B22" s="10" t="str"/>
       <x:c r="C22" s="11" t="str"/>
       <x:c r="D22" s="25"/>
+      <x:c r="E22" s="26"/>
     </x:row>
     <x:row r="23" ht="23" customHeight="1">
       <x:c r="A23" s="9" t="str"/>
       <x:c r="B23" s="10" t="str"/>
       <x:c r="C23" s="11" t="str"/>
       <x:c r="D23" s="25"/>
+      <x:c r="E23" s="26"/>
     </x:row>
     <x:row r="24" ht="23" customHeight="1">
       <x:c r="A24" s="9" t="str"/>
       <x:c r="B24" s="10" t="str"/>
       <x:c r="C24" s="11" t="str"/>
       <x:c r="D24" s="25"/>
+      <x:c r="E24" s="26"/>
     </x:row>
     <x:row r="25" ht="23" customHeight="1">
       <x:c r="A25" s="9" t="str"/>
       <x:c r="B25" s="10" t="str"/>
       <x:c r="C25" s="11" t="str"/>
       <x:c r="D25" s="25"/>
+      <x:c r="E25" s="26"/>
     </x:row>
     <x:row r="26" ht="23" customHeight="1">
       <x:c r="A26" s="9" t="str"/>
       <x:c r="B26" s="10" t="str"/>
       <x:c r="C26" s="11" t="str"/>
       <x:c r="D26" s="25"/>
+      <x:c r="E26" s="26"/>
     </x:row>
     <x:row r="27" ht="23" customHeight="1">
       <x:c r="A27" s="9" t="str"/>
       <x:c r="B27" s="10" t="str"/>
       <x:c r="C27" s="11" t="str"/>
       <x:c r="D27" s="25"/>
+      <x:c r="E27" s="26"/>
     </x:row>
     <x:row r="28" ht="23" customHeight="1">
       <x:c r="A28" s="9" t="str"/>
       <x:c r="B28" s="10" t="str"/>
       <x:c r="C28" s="11" t="str"/>
       <x:c r="D28" s="25"/>
+      <x:c r="E28" s="26"/>
     </x:row>
     <x:row r="29" ht="23" customHeight="1">
       <x:c r="A29" s="9" t="str"/>
       <x:c r="B29" s="10" t="str"/>
       <x:c r="C29" s="11" t="str"/>
       <x:c r="D29" s="25"/>
+      <x:c r="E29" s="26"/>
     </x:row>
     <x:row r="30" ht="23" customHeight="1">
       <x:c r="A30" s="9" t="str"/>
       <x:c r="B30" s="10" t="str"/>
       <x:c r="C30" s="11" t="str"/>
       <x:c r="D30" s="25"/>
+      <x:c r="E30" s="26"/>
     </x:row>
     <x:row r="31" ht="23" customHeight="1">
       <x:c r="A31" s="9" t="str"/>
       <x:c r="B31" s="10" t="str"/>
       <x:c r="C31" s="11" t="str"/>
       <x:c r="D31" s="25"/>
+      <x:c r="E31" s="26"/>
     </x:row>
     <x:row r="32" ht="23" customHeight="1">
       <x:c r="A32" s="9" t="str"/>
       <x:c r="B32" s="10" t="str"/>
       <x:c r="C32" s="11" t="str"/>
       <x:c r="D32" s="25"/>
+      <x:c r="E32" s="26"/>
     </x:row>
     <x:row r="33" ht="23" customHeight="1">
       <x:c r="A33" s="9" t="str"/>
       <x:c r="B33" s="10" t="str"/>
       <x:c r="C33" s="11" t="str"/>
       <x:c r="D33" s="25"/>
+      <x:c r="E33" s="26"/>
     </x:row>
     <x:row r="34" ht="23" customHeight="1">
       <x:c r="A34" s="9" t="str"/>
       <x:c r="B34" s="10" t="str"/>
       <x:c r="C34" s="11" t="str"/>
       <x:c r="D34" s="25"/>
+      <x:c r="E34" s="26"/>
     </x:row>
     <x:row r="35" ht="23" customHeight="1">
       <x:c r="A35" s="9" t="str"/>
       <x:c r="B35" s="10" t="str"/>
       <x:c r="C35" s="11" t="str"/>
       <x:c r="D35" s="25"/>
+      <x:c r="E35" s="26"/>
     </x:row>
     <x:row r="36" ht="23" customHeight="1">
       <x:c r="A36" s="9" t="str"/>
       <x:c r="B36" s="10" t="str"/>
       <x:c r="C36" s="11" t="str"/>
       <x:c r="D36" s="25"/>
+      <x:c r="E36" s="26"/>
     </x:row>
     <x:row r="37" ht="23" customHeight="1">
       <x:c r="A37" s="9" t="str"/>
       <x:c r="B37" s="10" t="str"/>
       <x:c r="C37" s="11" t="str"/>
       <x:c r="D37" s="25"/>
+      <x:c r="E37" s="26"/>
     </x:row>
     <x:row r="38" ht="23" customHeight="1">
       <x:c r="A38" s="9" t="str"/>
       <x:c r="B38" s="10" t="str"/>
       <x:c r="C38" s="11" t="str"/>
       <x:c r="D38" s="25"/>
+      <x:c r="E38" s="26"/>
     </x:row>
     <x:row r="39" ht="23" customHeight="1">
       <x:c r="A39" s="9" t="str"/>
       <x:c r="B39" s="10" t="str"/>
       <x:c r="C39" s="11" t="str"/>
       <x:c r="D39" s="25"/>
+      <x:c r="E39" s="26"/>
     </x:row>
     <x:row r="40" ht="23" customHeight="1">
       <x:c r="A40" s="9" t="str"/>
       <x:c r="B40" s="10" t="str"/>
       <x:c r="C40" s="11" t="str"/>
       <x:c r="D40" s="25"/>
+      <x:c r="E40" s="26"/>
     </x:row>
     <x:row r="41" ht="23" customHeight="1">
       <x:c r="A41" s="9" t="str"/>
       <x:c r="B41" s="10" t="str"/>
       <x:c r="C41" s="11" t="str"/>
       <x:c r="D41" s="25"/>
+      <x:c r="E41" s="26"/>
     </x:row>
     <x:row r="42" ht="23" customHeight="1">
       <x:c r="A42" s="9" t="str"/>
       <x:c r="B42" s="10" t="str"/>
       <x:c r="C42" s="11" t="str"/>
       <x:c r="D42" s="25"/>
+      <x:c r="E42" s="26"/>
     </x:row>
     <x:row r="43" ht="23" customHeight="1">
       <x:c r="A43" s="9" t="str"/>
       <x:c r="B43" s="10" t="str"/>
       <x:c r="C43" s="11" t="str"/>
       <x:c r="D43" s="25"/>
+      <x:c r="E43" s="26"/>
     </x:row>
     <x:row r="44" ht="23" customHeight="1">
       <x:c r="A44" s="9" t="str"/>
       <x:c r="B44" s="10" t="str"/>
       <x:c r="C44" s="11" t="str"/>
       <x:c r="D44" s="25"/>
+      <x:c r="E44" s="26"/>
     </x:row>
     <x:row r="45" ht="23" customHeight="1">
       <x:c r="A45" s="9" t="str"/>
       <x:c r="B45" s="10" t="str"/>
       <x:c r="C45" s="11" t="str"/>
       <x:c r="D45" s="25"/>
+      <x:c r="E45" s="26"/>
     </x:row>
     <x:row r="46" ht="23" customHeight="1">
       <x:c r="A46" s="9" t="str"/>
       <x:c r="B46" s="10" t="str"/>
       <x:c r="C46" s="11" t="str"/>
       <x:c r="D46" s="25"/>
+      <x:c r="E46" s="26"/>
     </x:row>
     <x:row r="47" ht="23" customHeight="1">
       <x:c r="A47" s="9" t="str"/>
       <x:c r="B47" s="10" t="str"/>
       <x:c r="C47" s="11" t="str"/>
       <x:c r="D47" s="25"/>
+      <x:c r="E47" s="26"/>
     </x:row>
     <x:row r="48" ht="23" customHeight="1">
       <x:c r="A48" s="9" t="str"/>
       <x:c r="B48" s="10" t="str"/>
       <x:c r="C48" s="11" t="str"/>
       <x:c r="D48" s="25"/>
+      <x:c r="E48" s="26"/>
     </x:row>
     <x:row r="49" ht="23" customHeight="1">
       <x:c r="A49" s="9" t="str"/>
       <x:c r="B49" s="10" t="str"/>
       <x:c r="C49" s="11" t="str"/>
       <x:c r="D49" s="25"/>
+      <x:c r="E49" s="26"/>
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="9" t="str"/>
       <x:c r="B50" s="10" t="str"/>
       <x:c r="C50" s="11" t="str"/>
       <x:c r="D50" s="25"/>
+      <x:c r="E50" s="26"/>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="9" t="str"/>
       <x:c r="B51" s="10" t="str"/>
       <x:c r="C51" s="11" t="str"/>
       <x:c r="D51" s="25"/>
+      <x:c r="E51" s="26"/>
+    </x:row>
+    <x:row r="52">
+      <x:c r="E52" s="26"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="E53" s="26"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="E54" s="26"/>
+    </x:row>
+    <x:row r="55">
+      <x:c r="E55" s="26"/>
+    </x:row>
+    <x:row r="56">
+      <x:c r="E56" s="26"/>
+    </x:row>
+    <x:row r="57">
+      <x:c r="E57" s="26"/>
+    </x:row>
+    <x:row r="58">
+      <x:c r="E58" s="26"/>
+    </x:row>
+    <x:row r="59">
+      <x:c r="E59" s="26"/>
+    </x:row>
+    <x:row r="60">
+      <x:c r="E60" s="26"/>
+    </x:row>
+    <x:row r="61">
+      <x:c r="E61" s="26"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="E62" s="26"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="E63" s="26"/>
+    </x:row>
+    <x:row r="64">
+      <x:c r="E64" s="26"/>
+    </x:row>
+    <x:row r="65">
+      <x:c r="E65" s="26"/>
+    </x:row>
+    <x:row r="66">
+      <x:c r="E66" s="26"/>
+    </x:row>
+    <x:row r="67">
+      <x:c r="E67" s="26"/>
+    </x:row>
+    <x:row r="68">
+      <x:c r="E68" s="26"/>
+    </x:row>
+    <x:row r="69">
+      <x:c r="E69" s="26"/>
+    </x:row>
+    <x:row r="70">
+      <x:c r="E70" s="26"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="E71" s="26"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="E72" s="26"/>
+    </x:row>
+    <x:row r="73">
+      <x:c r="E73" s="26"/>
+    </x:row>
+    <x:row r="74">
+      <x:c r="E74" s="26"/>
+    </x:row>
+    <x:row r="75">
+      <x:c r="E75" s="26"/>
+    </x:row>
+    <x:row r="76">
+      <x:c r="E76" s="26"/>
+    </x:row>
+    <x:row r="77">
+      <x:c r="E77" s="26"/>
+    </x:row>
+    <x:row r="78">
+      <x:c r="E78" s="26"/>
+    </x:row>
+    <x:row r="79">
+      <x:c r="E79" s="26"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="E80" s="26"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="E81" s="26"/>
+    </x:row>
+    <x:row r="82">
+      <x:c r="E82" s="26"/>
+    </x:row>
+    <x:row r="83">
+      <x:c r="E83" s="26"/>
+    </x:row>
+    <x:row r="84">
+      <x:c r="E84" s="26"/>
+    </x:row>
+    <x:row r="85">
+      <x:c r="E85" s="26"/>
+    </x:row>
+    <x:row r="86">
+      <x:c r="E86" s="26"/>
+    </x:row>
+    <x:row r="87">
+      <x:c r="E87" s="26"/>
+    </x:row>
+    <x:row r="88">
+      <x:c r="E88" s="26"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="E89" s="26"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="E90" s="26"/>
+    </x:row>
+    <x:row r="91">
+      <x:c r="E91" s="26"/>
+    </x:row>
+    <x:row r="92">
+      <x:c r="E92" s="26"/>
+    </x:row>
+    <x:row r="93">
+      <x:c r="E93" s="26"/>
+    </x:row>
+    <x:row r="94">
+      <x:c r="E94" s="26"/>
+    </x:row>
+    <x:row r="95">
+      <x:c r="E95" s="26"/>
+    </x:row>
+    <x:row r="96">
+      <x:c r="E96" s="26"/>
+    </x:row>
+    <x:row r="97">
+      <x:c r="E97" s="26"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="E98" s="26"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="E99" s="26"/>
+    </x:row>
+    <x:row r="100">
+      <x:c r="E100" s="26"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">

</xml_diff>